<commit_message>
062425 - update Ton to Tony in skins page week 7
</commit_message>
<xml_diff>
--- a/public/results/2025/Week 7 Skins.xlsx
+++ b/public/results/2025/Week 7 Skins.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="8_{DBBB26E3-A62B-4C64-B177-E34D2F1A43A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6EAD785F-3944-4B43-BE06-68E9C61988DB}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="8_{DBBB26E3-A62B-4C64-B177-E34D2F1A43A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24DF8014-0358-4F9B-A5F0-CBC41013F47E}"/>
   <bookViews>
-    <workbookView xWindow="43470" yWindow="3600" windowWidth="26730" windowHeight="18000" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
+    <workbookView xWindow="7515" yWindow="2640" windowWidth="26730" windowHeight="18000" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 7 Skins" sheetId="1" r:id="rId1"/>
@@ -83,9 +83,6 @@
     <t>Mark Y</t>
   </si>
   <si>
-    <t>Ton A</t>
-  </si>
-  <si>
     <t>Ryan M</t>
   </si>
   <si>
@@ -111,6 +108,9 @@
   </si>
   <si>
     <t>Tony (.5)</t>
+  </si>
+  <si>
+    <t>Tony A</t>
   </si>
 </sst>
 </file>
@@ -658,12 +658,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -676,6 +670,36 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
@@ -684,30 +708,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1051,28 +1051,28 @@
   <dimension ref="A1:O31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.140625" style="44"/>
-    <col min="3" max="11" width="8.7109375" style="44" customWidth="1"/>
-    <col min="12" max="12" width="4.28515625" style="44" customWidth="1"/>
-    <col min="13" max="13" width="5.85546875" style="44" customWidth="1"/>
-    <col min="14" max="15" width="6.5703125" style="44" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="44"/>
+    <col min="1" max="2" width="9.140625" style="39"/>
+    <col min="3" max="11" width="8.7109375" style="39" customWidth="1"/>
+    <col min="12" max="12" width="4.28515625" style="39" customWidth="1"/>
+    <col min="13" max="13" width="5.85546875" style="39" customWidth="1"/>
+    <col min="14" max="15" width="6.5703125" style="39" customWidth="1"/>
+    <col min="16" max="16384" width="9.140625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>1</v>
@@ -1083,7 +1083,7 @@
       </c>
     </row>
     <row r="2" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="40" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="5" t="s">
@@ -1116,15 +1116,15 @@
       <c r="K2" s="6">
         <v>9</v>
       </c>
-      <c r="L2" s="40" t="s">
-        <v>22</v>
+      <c r="L2" s="48" t="s">
+        <v>21</v>
       </c>
       <c r="M2" s="7"/>
       <c r="N2" s="8"/>
       <c r="O2" s="9"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="46"/>
+      <c r="A3" s="41"/>
       <c r="B3" s="10" t="s">
         <v>5</v>
       </c>
@@ -1155,13 +1155,13 @@
       <c r="K3" s="11">
         <v>5</v>
       </c>
-      <c r="L3" s="41"/>
+      <c r="L3" s="49"/>
       <c r="M3" s="12"/>
       <c r="N3" s="13"/>
       <c r="O3" s="13"/>
     </row>
     <row r="4" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="47"/>
+      <c r="A4" s="42"/>
       <c r="B4" s="14" t="s">
         <v>6</v>
       </c>
@@ -1192,13 +1192,13 @@
       <c r="K4" s="15">
         <v>2</v>
       </c>
-      <c r="L4" s="42"/>
+      <c r="L4" s="50"/>
       <c r="M4" s="12"/>
       <c r="N4" s="13"/>
       <c r="O4" s="13"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="48" t="s">
+      <c r="A5" s="43" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="16"/>
@@ -1229,13 +1229,13 @@
       <c r="K5" s="17">
         <v>4</v>
       </c>
-      <c r="L5" s="43"/>
+      <c r="L5" s="38"/>
       <c r="M5" s="19"/>
       <c r="N5" s="20"/>
       <c r="O5" s="20"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="49"/>
+      <c r="A6" s="44"/>
       <c r="B6" s="21"/>
       <c r="C6" s="21">
         <v>2</v>
@@ -1273,7 +1273,7 @@
       <c r="O6" s="20"/>
     </row>
     <row r="7" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="50"/>
+      <c r="A7" s="45"/>
       <c r="B7" s="23"/>
       <c r="C7" s="24">
         <f>C5-C6</f>
@@ -1323,8 +1323,8 @@
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="48" t="s">
-        <v>15</v>
+      <c r="A8" s="43" t="s">
+        <v>24</v>
       </c>
       <c r="B8" s="16"/>
       <c r="C8" s="16">
@@ -1354,13 +1354,13 @@
       <c r="K8" s="17">
         <v>7</v>
       </c>
-      <c r="L8" s="43"/>
+      <c r="L8" s="38"/>
       <c r="M8" s="19"/>
       <c r="N8" s="20"/>
       <c r="O8" s="13"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="49"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="21"/>
       <c r="C9" s="21">
         <v>2</v>
@@ -1398,7 +1398,7 @@
       <c r="O9" s="13"/>
     </row>
     <row r="10" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="50"/>
+      <c r="A10" s="45"/>
       <c r="B10" s="23"/>
       <c r="C10" s="23">
         <f>C8-C9</f>
@@ -1448,8 +1448,8 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="48" t="s">
-        <v>16</v>
+      <c r="A11" s="43" t="s">
+        <v>15</v>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="16">
@@ -1479,13 +1479,13 @@
       <c r="K11" s="17">
         <v>6</v>
       </c>
-      <c r="L11" s="43"/>
+      <c r="L11" s="38"/>
       <c r="M11" s="19"/>
       <c r="N11" s="20"/>
       <c r="O11" s="13"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="49"/>
+      <c r="A12" s="44"/>
       <c r="B12" s="21"/>
       <c r="C12" s="21">
         <v>1</v>
@@ -1523,7 +1523,7 @@
       <c r="O12" s="13"/>
     </row>
     <row r="13" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="50"/>
+      <c r="A13" s="45"/>
       <c r="B13" s="23"/>
       <c r="C13" s="24">
         <f>C11-C12</f>
@@ -1573,8 +1573,8 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="48" t="s">
-        <v>17</v>
+      <c r="A14" s="43" t="s">
+        <v>16</v>
       </c>
       <c r="B14" s="16"/>
       <c r="C14" s="16">
@@ -1604,13 +1604,13 @@
       <c r="K14" s="17">
         <v>6</v>
       </c>
-      <c r="L14" s="43"/>
+      <c r="L14" s="38"/>
       <c r="M14" s="19"/>
       <c r="N14" s="20"/>
       <c r="O14" s="13"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="49"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="21"/>
       <c r="C15" s="21">
         <v>2</v>
@@ -1648,7 +1648,7 @@
       <c r="O15" s="13"/>
     </row>
     <row r="16" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="50"/>
+      <c r="A16" s="45"/>
       <c r="B16" s="23"/>
       <c r="C16" s="24">
         <f>C14-C15</f>
@@ -1698,8 +1698,8 @@
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="48" t="s">
-        <v>18</v>
+      <c r="A17" s="43" t="s">
+        <v>17</v>
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="16">
@@ -1729,13 +1729,13 @@
       <c r="K17" s="17">
         <v>6</v>
       </c>
-      <c r="L17" s="43"/>
+      <c r="L17" s="38"/>
       <c r="M17" s="19"/>
       <c r="N17" s="20"/>
       <c r="O17" s="13"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="49"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="21"/>
       <c r="C18" s="21">
         <v>1</v>
@@ -1773,7 +1773,7 @@
       <c r="O18" s="13"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="50"/>
+      <c r="A19" s="45"/>
       <c r="B19" s="23"/>
       <c r="C19" s="23">
         <f>C17-C18</f>
@@ -1823,8 +1823,8 @@
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="48" t="s">
-        <v>19</v>
+      <c r="A20" s="43" t="s">
+        <v>18</v>
       </c>
       <c r="B20" s="16"/>
       <c r="C20" s="16">
@@ -1854,13 +1854,13 @@
       <c r="K20" s="17">
         <v>6</v>
       </c>
-      <c r="L20" s="43"/>
+      <c r="L20" s="38"/>
       <c r="M20" s="19"/>
       <c r="N20" s="20"/>
       <c r="O20" s="13"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="49"/>
+      <c r="A21" s="44"/>
       <c r="B21" s="21"/>
       <c r="C21" s="21">
         <v>1</v>
@@ -1898,7 +1898,7 @@
       <c r="O21" s="13"/>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="50"/>
+      <c r="A22" s="45"/>
       <c r="B22" s="23"/>
       <c r="C22" s="23">
         <f>C20-C21</f>
@@ -1946,8 +1946,8 @@
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="48" t="s">
-        <v>20</v>
+      <c r="A23" s="43" t="s">
+        <v>19</v>
       </c>
       <c r="B23" s="16"/>
       <c r="C23" s="16">
@@ -1977,13 +1977,13 @@
       <c r="K23" s="17">
         <v>7</v>
       </c>
-      <c r="L23" s="43"/>
+      <c r="L23" s="38"/>
       <c r="M23" s="19"/>
       <c r="N23" s="20"/>
       <c r="O23" s="13"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="49"/>
+      <c r="A24" s="44"/>
       <c r="B24" s="21"/>
       <c r="C24" s="21">
         <v>3</v>
@@ -2021,7 +2021,7 @@
       <c r="O24" s="13"/>
     </row>
     <row r="25" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="50"/>
+      <c r="A25" s="45"/>
       <c r="B25" s="23"/>
       <c r="C25" s="24">
         <f>C23-C24</f>
@@ -2071,8 +2071,8 @@
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="48" t="s">
-        <v>21</v>
+      <c r="A26" s="43" t="s">
+        <v>20</v>
       </c>
       <c r="B26" s="16"/>
       <c r="C26" s="16">
@@ -2108,7 +2108,7 @@
       <c r="O26" s="13"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="49"/>
+      <c r="A27" s="44"/>
       <c r="B27" s="21"/>
       <c r="C27" s="21">
         <v>2</v>
@@ -2146,7 +2146,7 @@
       <c r="O27" s="13"/>
     </row>
     <row r="28" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="50"/>
+      <c r="A28" s="45"/>
       <c r="B28" s="23"/>
       <c r="C28" s="23">
         <f>C26-C27</f>
@@ -2213,40 +2213,40 @@
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="32"/>
       <c r="B30" s="32"/>
-      <c r="C30" s="39" t="s">
+      <c r="C30" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="D30" s="39" t="s">
+      <c r="D30" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="E30" s="39" t="s">
+      <c r="E30" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="F30" s="39" t="s">
+      <c r="F30" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="G30" s="39" t="s">
+      <c r="G30" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="H30" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="I30" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="J30" s="39" t="s">
+      <c r="H30" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="I30" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="J30" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="K30" s="39" t="s">
+      <c r="K30" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="L30" s="39"/>
-      <c r="M30" s="36"/>
-      <c r="N30" s="37">
+      <c r="L30" s="37"/>
+      <c r="M30" s="34"/>
+      <c r="N30" s="35">
         <f>SUM(N7:N29)</f>
         <v>39.96</v>
       </c>
-      <c r="O30" s="38">
+      <c r="O30" s="36">
         <f>SUM(O7:O29)</f>
         <v>39</v>
       </c>
@@ -2254,27 +2254,27 @@
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="32"/>
       <c r="B31" s="32"/>
-      <c r="C31" s="39"/>
-      <c r="D31" s="39"/>
-      <c r="E31" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F31" s="39"/>
-      <c r="G31" s="39"/>
-      <c r="H31" s="39" t="s">
+      <c r="C31" s="37"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="F31" s="37"/>
+      <c r="G31" s="37"/>
+      <c r="H31" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="I31" s="39" t="s">
+      <c r="I31" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="J31" s="39" t="s">
+      <c r="J31" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="K31" s="39"/>
-      <c r="L31" s="39"/>
-      <c r="M31" s="36"/>
-      <c r="N31" s="39"/>
-      <c r="O31" s="39"/>
+      <c r="K31" s="37"/>
+      <c r="L31" s="37"/>
+      <c r="M31" s="34"/>
+      <c r="N31" s="37"/>
+      <c r="O31" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
062425 - updated week 7 skins spreadsheet with Score/Strokes/Net labels
</commit_message>
<xml_diff>
--- a/public/results/2025/Week 7 Skins.xlsx
+++ b/public/results/2025/Week 7 Skins.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="8_{DBBB26E3-A62B-4C64-B177-E34D2F1A43A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24DF8014-0358-4F9B-A5F0-CBC41013F47E}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="8_{DBBB26E3-A62B-4C64-B177-E34D2F1A43A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00FCE3B6-7C91-4C88-B84D-7D8AA5376D69}"/>
   <bookViews>
-    <workbookView xWindow="7515" yWindow="2640" windowWidth="26730" windowHeight="18000" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
+    <workbookView xWindow="7170" yWindow="2295" windowWidth="26730" windowHeight="18000" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 7 Skins" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="28">
   <si>
     <t>Skins ($40) $4.44/hole</t>
   </si>
@@ -111,6 +111,15 @@
   </si>
   <si>
     <t>Tony A</t>
+  </si>
+  <si>
+    <t>Score</t>
+  </si>
+  <si>
+    <t>Strokes</t>
+  </si>
+  <si>
+    <t>Net</t>
   </si>
 </sst>
 </file>
@@ -120,7 +129,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -180,6 +189,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -557,7 +572,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -708,6 +723,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1052,7 +1076,11 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="39"/>
-    <col min="3" max="11" width="8.7109375" style="39" customWidth="1"/>
+    <col min="3" max="3" width="7.42578125" style="39" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" style="39" customWidth="1"/>
+    <col min="5" max="5" width="10" style="39" customWidth="1"/>
+    <col min="6" max="6" width="7.42578125" style="39" customWidth="1"/>
+    <col min="7" max="11" width="8.7109375" style="39" customWidth="1"/>
     <col min="12" max="12" width="4.28515625" style="39" customWidth="1"/>
     <col min="13" max="13" width="5.85546875" style="39" customWidth="1"/>
     <col min="14" max="15" width="6.5703125" style="39" customWidth="1"/>
@@ -1201,7 +1229,9 @@
       <c r="A5" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="16"/>
+      <c r="B5" s="51" t="s">
+        <v>25</v>
+      </c>
       <c r="C5" s="16">
         <v>5</v>
       </c>
@@ -1236,7 +1266,9 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="44"/>
-      <c r="B6" s="21"/>
+      <c r="B6" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="C6" s="21">
         <v>2</v>
       </c>
@@ -1274,7 +1306,9 @@
     </row>
     <row r="7" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="45"/>
-      <c r="B7" s="23"/>
+      <c r="B7" s="53" t="s">
+        <v>27</v>
+      </c>
       <c r="C7" s="24">
         <f>C5-C6</f>
         <v>3</v>
@@ -1326,7 +1360,9 @@
       <c r="A8" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="16"/>
+      <c r="B8" s="51" t="s">
+        <v>25</v>
+      </c>
       <c r="C8" s="16">
         <v>6</v>
       </c>
@@ -1361,7 +1397,9 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="44"/>
-      <c r="B9" s="21"/>
+      <c r="B9" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="C9" s="21">
         <v>2</v>
       </c>
@@ -1399,7 +1437,9 @@
     </row>
     <row r="10" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="45"/>
-      <c r="B10" s="23"/>
+      <c r="B10" s="53" t="s">
+        <v>27</v>
+      </c>
       <c r="C10" s="23">
         <f>C8-C9</f>
         <v>4</v>
@@ -1451,7 +1491,9 @@
       <c r="A11" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="16"/>
+      <c r="B11" s="51" t="s">
+        <v>25</v>
+      </c>
       <c r="C11" s="16">
         <v>4</v>
       </c>
@@ -1486,7 +1528,9 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="44"/>
-      <c r="B12" s="21"/>
+      <c r="B12" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="C12" s="21">
         <v>1</v>
       </c>
@@ -1524,7 +1568,9 @@
     </row>
     <row r="13" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="45"/>
-      <c r="B13" s="23"/>
+      <c r="B13" s="53" t="s">
+        <v>27</v>
+      </c>
       <c r="C13" s="24">
         <f>C11-C12</f>
         <v>3</v>
@@ -1576,7 +1622,9 @@
       <c r="A14" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="16"/>
+      <c r="B14" s="51" t="s">
+        <v>25</v>
+      </c>
       <c r="C14" s="16">
         <v>5</v>
       </c>
@@ -1611,7 +1659,9 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="44"/>
-      <c r="B15" s="21"/>
+      <c r="B15" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="C15" s="21">
         <v>2</v>
       </c>
@@ -1649,7 +1699,9 @@
     </row>
     <row r="16" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="45"/>
-      <c r="B16" s="23"/>
+      <c r="B16" s="53" t="s">
+        <v>27</v>
+      </c>
       <c r="C16" s="24">
         <f>C14-C15</f>
         <v>3</v>
@@ -1701,7 +1753,9 @@
       <c r="A17" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="51" t="s">
+        <v>25</v>
+      </c>
       <c r="C17" s="16">
         <v>6</v>
       </c>
@@ -1736,7 +1790,9 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="44"/>
-      <c r="B18" s="21"/>
+      <c r="B18" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="C18" s="21">
         <v>1</v>
       </c>
@@ -1774,7 +1830,9 @@
     </row>
     <row r="19" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="45"/>
-      <c r="B19" s="23"/>
+      <c r="B19" s="53" t="s">
+        <v>27</v>
+      </c>
       <c r="C19" s="23">
         <f>C17-C18</f>
         <v>5</v>
@@ -1826,7 +1884,9 @@
       <c r="A20" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="16"/>
+      <c r="B20" s="51" t="s">
+        <v>25</v>
+      </c>
       <c r="C20" s="16">
         <v>5</v>
       </c>
@@ -1861,7 +1921,9 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="44"/>
-      <c r="B21" s="21"/>
+      <c r="B21" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="C21" s="21">
         <v>1</v>
       </c>
@@ -1899,7 +1961,9 @@
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="45"/>
-      <c r="B22" s="23"/>
+      <c r="B22" s="53" t="s">
+        <v>27</v>
+      </c>
       <c r="C22" s="23">
         <f>C20-C21</f>
         <v>4</v>
@@ -1949,7 +2013,9 @@
       <c r="A23" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="B23" s="16"/>
+      <c r="B23" s="51" t="s">
+        <v>25</v>
+      </c>
       <c r="C23" s="16">
         <v>6</v>
       </c>
@@ -1984,7 +2050,9 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="44"/>
-      <c r="B24" s="21"/>
+      <c r="B24" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="C24" s="21">
         <v>3</v>
       </c>
@@ -2022,7 +2090,9 @@
     </row>
     <row r="25" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="45"/>
-      <c r="B25" s="23"/>
+      <c r="B25" s="53" t="s">
+        <v>27</v>
+      </c>
       <c r="C25" s="24">
         <f>C23-C24</f>
         <v>3</v>
@@ -2074,7 +2144,9 @@
       <c r="A26" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="B26" s="16"/>
+      <c r="B26" s="51" t="s">
+        <v>25</v>
+      </c>
       <c r="C26" s="16">
         <v>8</v>
       </c>
@@ -2109,7 +2181,9 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="44"/>
-      <c r="B27" s="21"/>
+      <c r="B27" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="C27" s="21">
         <v>2</v>
       </c>
@@ -2147,7 +2221,9 @@
     </row>
     <row r="28" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="45"/>
-      <c r="B28" s="23"/>
+      <c r="B28" s="53" t="s">
+        <v>27</v>
+      </c>
       <c r="C28" s="23">
         <f>C26-C27</f>
         <v>6</v>

</xml_diff>